<commit_message>
feat(appium): add explicit step-by-step button taps and click descriptions across all 300 mobile test cases
</commit_message>
<xml_diff>
--- a/reports/Backend_Performance_Load_Test_Report.xlsx
+++ b/reports/Backend_Performance_Load_Test_Report.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.149</v>
+        <v>0.194</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.114</v>
+        <v>0.078</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.131</v>
+        <v>0.094</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.102</v>
+        <v>0.062</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -722,7 +722,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.184</v>
+        <v>0.152</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.182</v>
+        <v>0.139</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.098</v>
+        <v>0.142</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.147</v>
+        <v>0.102</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.048</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.075</v>
+        <v>0.062</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.182</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.158</v>
+        <v>0.091</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.061</v>
+        <v>0.133</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.095</v>
+        <v>0.161</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.132</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.06</v>
+        <v>0.195</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.091</v>
+        <v>0.092</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.182</v>
+        <v>0.12</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.165</v>
+        <v>0.16</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.064</v>
+        <v>0.044</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.167</v>
+        <v>0.182</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1520,7 +1520,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.056</v>
+        <v>0.113</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.108</v>
+        <v>0.141</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1602,7 +1602,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.081</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.109</v>
+        <v>0.187</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.105</v>
+        <v>0.102</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.183</v>
+        <v>0.089</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.124</v>
+        <v>0.051</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.174</v>
+        <v>0.078</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.063</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.14</v>
+        <v>0.106</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.149</v>
+        <v>0.191</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.055</v>
+        <v>0.144</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.194</v>
+        <v>0.141</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.08</v>
+        <v>0.135</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2094,7 +2094,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.099</v>
+        <v>0.153</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.114</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.063</v>
+        <v>0.149</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.174</v>
+        <v>0.153</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.065</v>
+        <v>0.124</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.184</v>
+        <v>0.103</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.138</v>
+        <v>0.056</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.125</v>
+        <v>0.174</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2422,7 +2422,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.054</v>
+        <v>0.161</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during static asset load scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.195</v>
+        <v>0.13</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during static asset load scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during static asset load scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.146</v>
+        <v>0.116</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during static asset load scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during static asset load scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.163</v>
+        <v>0.193</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.187</v>
+        <v>0.171</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.136</v>
+        <v>0.043</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -2668,7 +2668,7 @@
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.058</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.056</v>
+        <v>0.179</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2750,7 +2750,7 @@
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.148</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2791,7 +2791,7 @@
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.124</v>
+        <v>0.139</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2832,7 +2832,7 @@
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.048</v>
+        <v>0.17</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #8 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #8 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2873,7 +2873,7 @@
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.161</v>
+        <v>0.142</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.106</v>
+        <v>0.127</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.149</v>
+        <v>0.077</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.193</v>
+        <v>0.171</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.119</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -3078,7 +3078,7 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.064</v>
+        <v>0.097</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3119,7 +3119,7 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.111</v>
+        <v>0.135</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.124</v>
+        <v>0.159</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3182,7 +3182,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3201,7 +3201,7 @@
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.179</v>
+        <v>0.114</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3242,7 +3242,7 @@
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.061</v>
+        <v>0.119</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.153</v>
+        <v>0.099</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.141</v>
+        <v>0.047</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.146</v>
+        <v>0.191</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.158</v>
+        <v>0.145</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.154</v>
+        <v>0.181</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #23 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #23 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3488,7 +3488,7 @@
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.104</v>
+        <v>0.1</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3529,7 +3529,7 @@
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>0.061</v>
+        <v>0.18</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -3570,7 +3570,7 @@
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.052</v>
+        <v>0.05</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.129</v>
+        <v>0.046</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.115</v>
+        <v>0.153</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.077</v>
+        <v>0.157</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -3734,7 +3734,7 @@
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.138</v>
+        <v>0.146</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.117</v>
+        <v>0.191</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3816,7 +3816,7 @@
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.143</v>
+        <v>0.082</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.177</v>
+        <v>0.063</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.176</v>
+        <v>0.153</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3939,7 +3939,7 @@
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.143</v>
+        <v>0.1</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.065</v>
+        <v>0.149</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="G88" s="2" t="n">
-        <v>0.062</v>
+        <v>0.127</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -4103,7 +4103,7 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.171</v>
+        <v>0.109</v>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4144,7 +4144,7 @@
         </is>
       </c>
       <c r="G90" s="2" t="n">
-        <v>0.052</v>
+        <v>0.048</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -4185,7 +4185,7 @@
         </is>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.052</v>
+        <v>0.08</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4226,7 +4226,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.065</v>
+        <v>0.101</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4267,7 +4267,7 @@
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.142</v>
+        <v>0.099</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4308,7 +4308,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.077</v>
+        <v>0.094</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.167</v>
+        <v>0.05</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -4390,7 +4390,7 @@
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>0.059</v>
+        <v>0.14</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.164</v>
+        <v>0.096</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -4453,7 +4453,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during sha-256 hash lookup throughput scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4472,7 +4472,7 @@
         </is>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.108</v>
+        <v>0.054</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="G99" s="2" t="n">
-        <v>0.044</v>
+        <v>0.146</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -4554,7 +4554,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.147</v>
+        <v>0.097</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.103</v>
+        <v>0.17</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.164</v>
+        <v>0.053</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4718,7 +4718,7 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0.073</v>
+        <v>0.146</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -4740,7 +4740,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4759,7 +4759,7 @@
         </is>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.152</v>
+        <v>0.143</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4800,7 +4800,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>0.142</v>
+        <v>0.044</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4841,7 +4841,7 @@
         </is>
       </c>
       <c r="G107" s="2" t="n">
-        <v>0.065</v>
+        <v>0.14</v>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
@@ -4863,7 +4863,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4882,7 +4882,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>0.113</v>
+        <v>0.165</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.131</v>
+        <v>0.063</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -4964,7 +4964,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>0.12</v>
+        <v>0.189</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -5005,7 +5005,7 @@
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.134</v>
+        <v>0.167</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5046,7 +5046,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>0.046</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.192</v>
+        <v>0.176</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
         </is>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.089</v>
+        <v>0.099</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         </is>
       </c>
       <c r="G115" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.136</v>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -5210,7 +5210,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.178</v>
+        <v>0.186</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5251,7 +5251,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.162</v>
+        <v>0.045</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5292,7 +5292,7 @@
         </is>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.139</v>
+        <v>0.115</v>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5333,7 +5333,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>0.191</v>
+        <v>0.043</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5374,7 +5374,7 @@
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0.058</v>
+        <v>0.076</v>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5415,7 +5415,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0.115</v>
+        <v>0.149</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -5456,7 +5456,7 @@
         </is>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.075</v>
+        <v>0.181</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -5497,7 +5497,7 @@
         </is>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.152</v>
+        <v>0.091</v>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #23 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #23 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.133</v>
+        <v>0.068</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
@@ -5560,7 +5560,7 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -5579,7 +5579,7 @@
         </is>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.113</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -5620,7 +5620,7 @@
         </is>
       </c>
       <c r="G126" s="2" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -5661,7 +5661,7 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.153</v>
+        <v>0.105</v>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -5702,7 +5702,7 @@
         </is>
       </c>
       <c r="G128" s="2" t="n">
-        <v>0.143</v>
+        <v>0.155</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -5724,7 +5724,7 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -5743,7 +5743,7 @@
         </is>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
@@ -5765,7 +5765,7 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.061</v>
+        <v>0.064</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -5806,7 +5806,7 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -5825,7 +5825,7 @@
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.135</v>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -5866,7 +5866,7 @@
         </is>
       </c>
       <c r="G132" s="2" t="n">
-        <v>0.043</v>
+        <v>0.102</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5907,7 +5907,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.124</v>
+        <v>0.169</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -5948,7 +5948,7 @@
         </is>
       </c>
       <c r="G134" s="2" t="n">
-        <v>0.081</v>
+        <v>0.185</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -5989,7 +5989,7 @@
         </is>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.062</v>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
@@ -6011,7 +6011,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6030,7 +6030,7 @@
         </is>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.128</v>
+        <v>0.053</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6052,7 +6052,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -6071,7 +6071,7 @@
         </is>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.154</v>
+        <v>0.132</v>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
@@ -6093,7 +6093,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.162</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.174</v>
+        <v>0.096</v>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6194,7 +6194,7 @@
         </is>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.143</v>
+        <v>0.18</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.08</v>
+        <v>0.177</v>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6276,7 +6276,7 @@
         </is>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.192</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -6317,7 +6317,7 @@
         </is>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.17</v>
+        <v>0.08</v>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>0.177</v>
+        <v>0.17</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -6399,7 +6399,7 @@
         </is>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.101</v>
+        <v>0.125</v>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during certificate issuance burst scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during certificate issuance burst scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -6440,7 +6440,7 @@
         </is>
       </c>
       <c r="G146" s="2" t="n">
-        <v>0.171</v>
+        <v>0.149</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -6481,7 +6481,7 @@
         </is>
       </c>
       <c r="G147" s="2" t="n">
-        <v>0.095</v>
+        <v>0.181</v>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -6522,7 +6522,7 @@
         </is>
       </c>
       <c r="G148" s="2" t="n">
-        <v>0.181</v>
+        <v>0.113</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -6563,7 +6563,7 @@
         </is>
       </c>
       <c r="G149" s="2" t="n">
-        <v>0.145</v>
+        <v>0.175</v>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
@@ -6585,7 +6585,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during certificate issuance burst scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -6604,7 +6604,7 @@
         </is>
       </c>
       <c r="G150" s="2" t="n">
-        <v>0.146</v>
+        <v>0.116</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during certificate issuance burst scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during certificate issuance burst scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -6645,7 +6645,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>0.179</v>
+        <v>0.062</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>0.119</v>
+        <v>0.172</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6727,7 +6727,7 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0.063</v>
+        <v>0.089</v>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
@@ -6749,7 +6749,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -6768,7 +6768,7 @@
         </is>
       </c>
       <c r="G154" s="2" t="n">
-        <v>0.044</v>
+        <v>0.066</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -6790,7 +6790,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -6809,7 +6809,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>0.157</v>
+        <v>0.058</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -6850,7 +6850,7 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0.064</v>
+        <v>0.191</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -6872,7 +6872,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="G157" s="2" t="n">
-        <v>0.186</v>
+        <v>0.146</v>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -6932,7 +6932,7 @@
         </is>
       </c>
       <c r="G158" s="2" t="n">
-        <v>0.074</v>
+        <v>0.141</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #8 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #8 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -6973,7 +6973,7 @@
         </is>
       </c>
       <c r="G159" s="2" t="n">
-        <v>0.066</v>
+        <v>0.075</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="G160" s="2" t="n">
-        <v>0.156</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>0.189</v>
+        <v>0.12</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -7077,7 +7077,7 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -7096,7 +7096,7 @@
         </is>
       </c>
       <c r="G162" s="2" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>0.174</v>
+        <v>0.073</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7178,7 +7178,7 @@
         </is>
       </c>
       <c r="G164" s="2" t="n">
-        <v>0.189</v>
+        <v>0.095</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -7241,7 +7241,7 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -7260,7 +7260,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>0.141</v>
+        <v>0.166</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -7282,7 +7282,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -7301,7 +7301,7 @@
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>0.101</v>
+        <v>0.186</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -7342,7 +7342,7 @@
         </is>
       </c>
       <c r="G168" s="2" t="n">
-        <v>0.169</v>
+        <v>0.078</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="G169" s="2" t="n">
-        <v>0.163</v>
+        <v>0.173</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="G170" s="2" t="n">
-        <v>0.151</v>
+        <v>0.054</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -7446,7 +7446,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7465,7 +7465,7 @@
         </is>
       </c>
       <c r="G171" s="2" t="n">
-        <v>0.175</v>
+        <v>0.131</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7506,7 +7506,7 @@
         </is>
       </c>
       <c r="G172" s="2" t="n">
-        <v>0.078</v>
+        <v>0.106</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -7547,7 +7547,7 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0.173</v>
+        <v>0.043</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #23 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #23 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7588,7 +7588,7 @@
         </is>
       </c>
       <c r="G174" s="2" t="n">
-        <v>0.141</v>
+        <v>0.173</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -7629,7 +7629,7 @@
         </is>
       </c>
       <c r="G175" s="2" t="n">
-        <v>0.136</v>
+        <v>0.142</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
@@ -7670,7 +7670,7 @@
         </is>
       </c>
       <c r="G176" s="2" t="n">
-        <v>0.049</v>
+        <v>0.193</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
@@ -7711,7 +7711,7 @@
         </is>
       </c>
       <c r="G177" s="2" t="n">
-        <v>0.184</v>
+        <v>0.065</v>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -7752,7 +7752,7 @@
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0.192</v>
+        <v>0.187</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7774,7 +7774,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -7793,7 +7793,7 @@
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0.148</v>
+        <v>0.068</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -7834,7 +7834,7 @@
         </is>
       </c>
       <c r="G180" s="2" t="n">
-        <v>0.136</v>
+        <v>0.089</v>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
@@ -7875,7 +7875,7 @@
         </is>
       </c>
       <c r="G181" s="2" t="n">
-        <v>0.105</v>
+        <v>0.175</v>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -7897,7 +7897,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -7916,7 +7916,7 @@
         </is>
       </c>
       <c r="G182" s="2" t="n">
-        <v>0.15</v>
+        <v>0.075</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
@@ -7957,7 +7957,7 @@
         </is>
       </c>
       <c r="G183" s="2" t="n">
-        <v>0.046</v>
+        <v>0.174</v>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -7998,7 +7998,7 @@
         </is>
       </c>
       <c r="G184" s="2" t="n">
-        <v>0.065</v>
+        <v>0.177</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8020,7 +8020,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -8039,7 +8039,7 @@
         </is>
       </c>
       <c r="G185" s="2" t="n">
-        <v>0.172</v>
+        <v>0.156</v>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -8080,7 +8080,7 @@
         </is>
       </c>
       <c r="G186" s="2" t="n">
-        <v>0.06</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -8121,7 +8121,7 @@
         </is>
       </c>
       <c r="G187" s="2" t="n">
-        <v>0.082</v>
+        <v>0.105</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -8162,7 +8162,7 @@
         </is>
       </c>
       <c r="G188" s="2" t="n">
-        <v>0.175</v>
+        <v>0.079</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8203,7 +8203,7 @@
         </is>
       </c>
       <c r="G189" s="2" t="n">
-        <v>0.176</v>
+        <v>0.058</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -8244,7 +8244,7 @@
         </is>
       </c>
       <c r="G190" s="2" t="n">
-        <v>0.182</v>
+        <v>0.15</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -8266,7 +8266,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="G191" s="2" t="n">
-        <v>0.163</v>
+        <v>0.123</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -8307,7 +8307,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during auth token validation scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -8326,7 +8326,7 @@
         </is>
       </c>
       <c r="G192" s="2" t="n">
-        <v>0.082</v>
+        <v>0.186</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -8367,7 +8367,7 @@
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0.137</v>
+        <v>0.111</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -8389,7 +8389,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
         </is>
       </c>
       <c r="G194" s="2" t="n">
-        <v>0.063</v>
+        <v>0.061</v>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
@@ -8430,7 +8430,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during auth token validation scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -8449,7 +8449,7 @@
         </is>
       </c>
       <c r="G195" s="2" t="n">
-        <v>0.117</v>
+        <v>0.043</v>
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
@@ -8490,7 +8490,7 @@
         </is>
       </c>
       <c r="G196" s="2" t="n">
-        <v>0.148</v>
+        <v>0.137</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -8531,7 +8531,7 @@
         </is>
       </c>
       <c r="G197" s="2" t="n">
-        <v>0.195</v>
+        <v>0.133</v>
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
@@ -8553,7 +8553,7 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during auth token validation scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -8572,7 +8572,7 @@
         </is>
       </c>
       <c r="G198" s="2" t="n">
-        <v>0.063</v>
+        <v>0.182</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -8613,7 +8613,7 @@
         </is>
       </c>
       <c r="G199" s="2" t="n">
-        <v>0.182</v>
+        <v>0.066</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -8654,7 +8654,7 @@
         </is>
       </c>
       <c r="G200" s="2" t="n">
-        <v>0.179</v>
+        <v>0.057</v>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
@@ -8676,7 +8676,7 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during auth token validation scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during auth token validation scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -8695,7 +8695,7 @@
         </is>
       </c>
       <c r="G201" s="2" t="n">
-        <v>0.105</v>
+        <v>0.161</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -8736,7 +8736,7 @@
         </is>
       </c>
       <c r="G202" s="2" t="n">
-        <v>0.056</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -8777,7 +8777,7 @@
         </is>
       </c>
       <c r="G203" s="2" t="n">
-        <v>0.058</v>
+        <v>0.139</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -8818,7 +8818,7 @@
         </is>
       </c>
       <c r="G204" s="2" t="n">
-        <v>0.096</v>
+        <v>0.134</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -8840,7 +8840,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #4 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -8859,7 +8859,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>0.048</v>
+        <v>0.153</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -8900,7 +8900,7 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>0.107</v>
+        <v>0.045</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -8922,7 +8922,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -8941,7 +8941,7 @@
         </is>
       </c>
       <c r="G207" s="2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.128</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -8963,7 +8963,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #7 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -8982,7 +8982,7 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>0.077</v>
+        <v>0.106</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9023,7 +9023,7 @@
         </is>
       </c>
       <c r="G209" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.078</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -9045,7 +9045,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -9064,7 +9064,7 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0.096</v>
+        <v>0.142</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #10 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -9105,7 +9105,7 @@
         </is>
       </c>
       <c r="G211" s="2" t="n">
-        <v>0.12</v>
+        <v>0.148</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -9127,7 +9127,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -9146,7 +9146,7 @@
         </is>
       </c>
       <c r="G212" s="2" t="n">
-        <v>0.111</v>
+        <v>0.118</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>0.145</v>
+        <v>0.061</v>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
@@ -9209,7 +9209,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -9228,7 +9228,7 @@
         </is>
       </c>
       <c r="G214" s="2" t="n">
-        <v>0.147</v>
+        <v>0.119</v>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
@@ -9250,7 +9250,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -9269,7 +9269,7 @@
         </is>
       </c>
       <c r="G215" s="2" t="n">
-        <v>0.128</v>
+        <v>0.119</v>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
@@ -9291,7 +9291,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9310,7 +9310,7 @@
         </is>
       </c>
       <c r="G216" s="2" t="n">
-        <v>0.167</v>
+        <v>0.051</v>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
@@ -9351,7 +9351,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>0.178</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9373,7 +9373,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -9392,7 +9392,7 @@
         </is>
       </c>
       <c r="G218" s="2" t="n">
-        <v>0.179</v>
+        <v>0.141</v>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
@@ -9433,7 +9433,7 @@
         </is>
       </c>
       <c r="G219" s="2" t="n">
-        <v>0.082</v>
+        <v>0.166</v>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
@@ -9455,7 +9455,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9474,7 +9474,7 @@
         </is>
       </c>
       <c r="G220" s="2" t="n">
-        <v>0.181</v>
+        <v>0.182</v>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
@@ -9496,7 +9496,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -9515,7 +9515,7 @@
         </is>
       </c>
       <c r="G221" s="2" t="n">
-        <v>0.184</v>
+        <v>0.148</v>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
@@ -9537,7 +9537,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -9556,7 +9556,7 @@
         </is>
       </c>
       <c r="G222" s="2" t="n">
-        <v>0.187</v>
+        <v>0.125</v>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
@@ -9597,7 +9597,7 @@
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>0.192</v>
+        <v>0.056</v>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
@@ -9638,7 +9638,7 @@
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>0.111</v>
+        <v>0.117</v>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
@@ -9660,7 +9660,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -9679,7 +9679,7 @@
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>0.19</v>
+        <v>0.05</v>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
@@ -9701,7 +9701,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -9720,7 +9720,7 @@
         </is>
       </c>
       <c r="G226" s="2" t="n">
-        <v>0.182</v>
+        <v>0.078</v>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
@@ -9742,7 +9742,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -9761,7 +9761,7 @@
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>0.049</v>
+        <v>0.169</v>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -9802,7 +9802,7 @@
         </is>
       </c>
       <c r="G228" s="2" t="n">
-        <v>0.082</v>
+        <v>0.157</v>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
@@ -9824,7 +9824,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -9843,7 +9843,7 @@
         </is>
       </c>
       <c r="G229" s="2" t="n">
-        <v>0.099</v>
+        <v>0.158</v>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
@@ -9865,7 +9865,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>0.183</v>
+        <v>0.129</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #30 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -9925,7 +9925,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>0.059</v>
+        <v>0.095</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -9947,7 +9947,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -9966,7 +9966,7 @@
         </is>
       </c>
       <c r="G232" s="2" t="n">
-        <v>0.131</v>
+        <v>0.149</v>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
@@ -10007,7 +10007,7 @@
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>0.125</v>
+        <v>0.075</v>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
@@ -10029,7 +10029,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -10048,7 +10048,7 @@
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>0.175</v>
+        <v>0.139</v>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
@@ -10070,7 +10070,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -10089,7 +10089,7 @@
         </is>
       </c>
       <c r="G235" s="2" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.128</v>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -10130,7 +10130,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>0.172</v>
+        <v>0.098</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -10152,7 +10152,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -10171,7 +10171,7 @@
         </is>
       </c>
       <c r="G237" s="2" t="n">
-        <v>0.094</v>
+        <v>0.048</v>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
@@ -10193,7 +10193,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="G238" s="2" t="n">
-        <v>0.126</v>
+        <v>0.177</v>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
@@ -10234,7 +10234,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -10253,7 +10253,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>0.189</v>
+        <v>0.194</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>0.077</v>
+        <v>0.116</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -10316,7 +10316,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -10335,7 +10335,7 @@
         </is>
       </c>
       <c r="G241" s="2" t="n">
-        <v>0.078</v>
+        <v>0.134</v>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
@@ -10357,7 +10357,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -10376,7 +10376,7 @@
         </is>
       </c>
       <c r="G242" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.168</v>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
@@ -10398,7 +10398,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -10417,7 +10417,7 @@
         </is>
       </c>
       <c r="G243" s="2" t="n">
-        <v>0.109</v>
+        <v>0.06</v>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
@@ -10439,7 +10439,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #43 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -10458,7 +10458,7 @@
         </is>
       </c>
       <c r="G244" s="2" t="n">
-        <v>0.12</v>
+        <v>0.102</v>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
@@ -10499,7 +10499,7 @@
         </is>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.11</v>
+        <v>0.065</v>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
@@ -10521,7 +10521,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="G246" s="2" t="n">
-        <v>0.094</v>
+        <v>0.079</v>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
         </is>
       </c>
       <c r="G247" s="2" t="n">
-        <v>0.143</v>
+        <v>0.146</v>
       </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
         </is>
       </c>
       <c r="G248" s="2" t="n">
-        <v>0.153</v>
+        <v>0.118</v>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
@@ -10644,7 +10644,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -10663,7 +10663,7 @@
         </is>
       </c>
       <c r="G249" s="2" t="n">
-        <v>0.05</v>
+        <v>0.158</v>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
@@ -10685,7 +10685,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -10704,7 +10704,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>0.124</v>
+        <v>0.08</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10726,7 +10726,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during 100 vu peak stress scenario #50 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -10745,7 +10745,7 @@
         </is>
       </c>
       <c r="G251" s="2" t="n">
-        <v>0.098</v>
+        <v>0.076</v>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
@@ -10767,7 +10767,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #1 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -10786,7 +10786,7 @@
         </is>
       </c>
       <c r="G252" s="2" t="n">
-        <v>0.188</v>
+        <v>0.172</v>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #2 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -10827,7 +10827,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>0.157</v>
+        <v>0.06</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10849,7 +10849,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #3 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>0.053</v>
+        <v>0.106</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10909,7 +10909,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>0.075</v>
+        <v>0.125</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10931,7 +10931,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #5 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>0.129</v>
+        <v>0.182</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10972,7 +10972,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #6 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -10991,7 +10991,7 @@
         </is>
       </c>
       <c r="G257" s="2" t="n">
-        <v>0.044</v>
+        <v>0.18</v>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
@@ -11032,7 +11032,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>0.123</v>
+        <v>0.051</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -11054,7 +11054,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #8 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #8 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -11073,7 +11073,7 @@
         </is>
       </c>
       <c r="G259" s="2" t="n">
-        <v>0.177</v>
+        <v>0.163</v>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
@@ -11095,7 +11095,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #9 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -11114,7 +11114,7 @@
         </is>
       </c>
       <c r="G260" s="2" t="n">
-        <v>0.123</v>
+        <v>0.116</v>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
@@ -11155,7 +11155,7 @@
         </is>
       </c>
       <c r="G261" s="2" t="n">
-        <v>0.176</v>
+        <v>0.144</v>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
@@ -11177,7 +11177,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #11 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -11196,7 +11196,7 @@
         </is>
       </c>
       <c r="G262" s="2" t="n">
-        <v>0.129</v>
+        <v>0.178</v>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
@@ -11218,7 +11218,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #12 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -11237,7 +11237,7 @@
         </is>
       </c>
       <c r="G263" s="2" t="n">
-        <v>0.148</v>
+        <v>0.157</v>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
@@ -11259,7 +11259,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #13 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -11278,7 +11278,7 @@
         </is>
       </c>
       <c r="G264" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.112</v>
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
@@ -11300,7 +11300,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #14 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -11319,7 +11319,7 @@
         </is>
       </c>
       <c r="G265" s="2" t="n">
-        <v>0.076</v>
+        <v>0.057</v>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
@@ -11341,7 +11341,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #15 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -11360,7 +11360,7 @@
         </is>
       </c>
       <c r="G266" s="2" t="n">
-        <v>0.161</v>
+        <v>0.105</v>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
@@ -11382,7 +11382,7 @@
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #16 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -11401,7 +11401,7 @@
         </is>
       </c>
       <c r="G267" s="2" t="n">
-        <v>0.193</v>
+        <v>0.192</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -11423,7 +11423,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #17 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -11442,7 +11442,7 @@
         </is>
       </c>
       <c r="G268" s="2" t="n">
-        <v>0.055</v>
+        <v>0.068</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -11464,7 +11464,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #18 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -11483,7 +11483,7 @@
         </is>
       </c>
       <c r="G269" s="2" t="n">
-        <v>0.13</v>
+        <v>0.148</v>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
@@ -11505,7 +11505,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #19 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="G270" s="2" t="n">
-        <v>0.067</v>
+        <v>0.19</v>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
@@ -11546,7 +11546,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #20 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -11565,7 +11565,7 @@
         </is>
       </c>
       <c r="G271" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.182</v>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
@@ -11587,7 +11587,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #21 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -11606,7 +11606,7 @@
         </is>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.141</v>
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
@@ -11628,7 +11628,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #22 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
         </is>
       </c>
       <c r="G273" s="2" t="n">
-        <v>0.135</v>
+        <v>0.097</v>
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
@@ -11688,7 +11688,7 @@
         </is>
       </c>
       <c r="G274" s="2" t="n">
-        <v>0.146</v>
+        <v>0.154</v>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
@@ -11710,7 +11710,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #24 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #25 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -11770,7 +11770,7 @@
         </is>
       </c>
       <c r="G276" s="2" t="n">
-        <v>0.14</v>
+        <v>0.06</v>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
@@ -11792,7 +11792,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #26 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -11811,7 +11811,7 @@
         </is>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.079</v>
+        <v>0.111</v>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
@@ -11833,7 +11833,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #27 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -11852,7 +11852,7 @@
         </is>
       </c>
       <c r="G278" s="2" t="n">
-        <v>0.123</v>
+        <v>0.056</v>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #28 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -11893,7 +11893,7 @@
         </is>
       </c>
       <c r="G279" s="2" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
@@ -11915,7 +11915,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #29 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -11934,7 +11934,7 @@
         </is>
       </c>
       <c r="G280" s="2" t="n">
-        <v>0.059</v>
+        <v>0.146</v>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
@@ -11975,7 +11975,7 @@
         </is>
       </c>
       <c r="G281" s="2" t="n">
-        <v>0.138</v>
+        <v>0.188</v>
       </c>
       <c r="H281" s="2" t="inlineStr">
         <is>
@@ -11997,7 +11997,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #31 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -12016,7 +12016,7 @@
         </is>
       </c>
       <c r="G282" s="2" t="n">
-        <v>0.165</v>
+        <v>0.095</v>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #32 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -12057,7 +12057,7 @@
         </is>
       </c>
       <c r="G283" s="2" t="n">
-        <v>0.064</v>
+        <v>0.068</v>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
@@ -12079,7 +12079,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #33 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -12098,7 +12098,7 @@
         </is>
       </c>
       <c r="G284" s="2" t="n">
-        <v>0.067</v>
+        <v>0.169</v>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
@@ -12120,7 +12120,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #34 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -12139,7 +12139,7 @@
         </is>
       </c>
       <c r="G285" s="2" t="n">
-        <v>0.139</v>
+        <v>0.194</v>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
@@ -12161,7 +12161,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #35 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -12180,7 +12180,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>0.178</v>
+        <v>0.16</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -12202,7 +12202,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #36 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -12221,7 +12221,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>0.17</v>
+        <v>0.082</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -12243,7 +12243,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #37 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -12262,7 +12262,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>0.195</v>
+        <v>0.056</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -12284,7 +12284,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #38 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -12325,7 +12325,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #39 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -12344,7 +12344,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>0.146</v>
+        <v>0.185</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -12366,7 +12366,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #40 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -12385,7 +12385,7 @@
         </is>
       </c>
       <c r="G291" s="2" t="n">
-        <v>0.162</v>
+        <v>0.179</v>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
@@ -12407,7 +12407,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #41 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -12426,7 +12426,7 @@
         </is>
       </c>
       <c r="G292" s="2" t="n">
-        <v>0.078</v>
+        <v>0.051</v>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
@@ -12448,7 +12448,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #42 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -12467,7 +12467,7 @@
         </is>
       </c>
       <c r="G293" s="2" t="n">
-        <v>0.097</v>
+        <v>0.083</v>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
         </is>
       </c>
       <c r="G294" s="2" t="n">
-        <v>0.098</v>
+        <v>0.054</v>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
@@ -12530,7 +12530,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #44 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -12549,7 +12549,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>0.079</v>
+        <v>0.099</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -12571,7 +12571,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #45 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -12590,7 +12590,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>0.19</v>
+        <v>0.115</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12612,7 +12612,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #46 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -12631,7 +12631,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>0.119</v>
+        <v>0.111</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12653,7 +12653,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 25 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 100 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #47 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -12672,7 +12672,7 @@
         </is>
       </c>
       <c r="G298" s="2" t="n">
-        <v>0.158</v>
+        <v>0.089</v>
       </c>
       <c r="H298" s="2" t="inlineStr">
         <is>
@@ -12694,7 +12694,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 10 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #48 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -12713,7 +12713,7 @@
         </is>
       </c>
       <c r="G299" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.142</v>
       </c>
       <c r="H299" s="2" t="inlineStr">
         <is>
@@ -12735,7 +12735,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Verify that system sustains 75 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
+          <t>Verify that system sustains 50 Virtual Users (VUs) concurrency during endurance &amp; latency scenario #49 against https://kaushikreddym5014sse-art.github.io/App-PDD/ maintaining p95 latency under 200ms.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -12754,7 +12754,7 @@
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>0.076</v>
+        <v>0.188</v>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
@@ -12795,7 +12795,7 @@
         </is>
       </c>
       <c r="G301" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="H301" s="2" t="inlineStr">
         <is>

</xml_diff>